<commit_message>
Fixed and updated the locators
</commit_message>
<xml_diff>
--- a/SmartHospitalTesting/src/test/resources/test_datas/BloodIssueValid.xlsx
+++ b/SmartHospitalTesting/src/test/resources/test_datas/BloodIssueValid.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{58C881FF-BCC3-4263-A4C3-A36929CAFD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{DE630C91-C98E-47B7-8EDC-AAE335B6667A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidDetails" sheetId="1" r:id="rId1"/>
@@ -401,7 +401,7 @@
     </row>
     <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
-        <v>531</v>
+        <v>1152</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>

</xml_diff>